<commit_message>
V1.4 - Agrega nombres integrantes: Felipe De Goyeneche y Maximiliano Masferrer
</commit_message>
<xml_diff>
--- a/pruebas/casos_prueba.xlsx
+++ b/pruebas/casos_prueba.xlsx
@@ -142,7 +142,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -192,11 +192,99 @@
         <color rgb="00003366"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00003366"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00003366"/>
+      </right>
+      <top style="thin">
+        <color rgb="00003366"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00003366"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00003366"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00003366"/>
+      </right>
+      <top style="thin">
+        <color rgb="00003366"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00003366"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -255,6 +343,10 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1039,6 +1131,14 @@
           <t>⚠ Columna 'Resultado obtenido' (fondo amarillo): completar con el resultado real observado al ejecutar cada caso sobre el prototipo Figma  |  Columna 'Evidencia': adjuntar captura de pantalla o indicar el nombre del archivo de imagen</t>
         </is>
       </c>
+      <c r="B11" s="20" t="n"/>
+      <c r="C11" s="20" t="n"/>
+      <c r="D11" s="20" t="n"/>
+      <c r="E11" s="20" t="n"/>
+      <c r="F11" s="20" t="n"/>
+      <c r="G11" s="20" t="n"/>
+      <c r="H11" s="20" t="n"/>
+      <c r="I11" s="21" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1132,7 +1232,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>[Integrante 1]</t>
+          <t>F. De Goyeneche</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -1169,7 +1269,7 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>[Integrante 2]</t>
+          <t>M. Masferrer</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
@@ -1206,7 +1306,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>[Integrante 3]</t>
+          <t>F. De Goyeneche</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -1378,6 +1478,9 @@
           <t>OBJETIVO</t>
         </is>
       </c>
+      <c r="B2" s="22" t="n"/>
+      <c r="C2" s="22" t="n"/>
+      <c r="D2" s="23" t="n"/>
     </row>
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -1385,6 +1488,9 @@
           <t>Verificar que el prototipo funcional del Sistema de Aduana cumple todos los requisitos funcionales y no funcionales definidos en el caso, aplicando el modelo de calidad ISO9126 bajo el marco ISO25000.</t>
         </is>
       </c>
+      <c r="B3" s="22" t="n"/>
+      <c r="C3" s="22" t="n"/>
+      <c r="D3" s="23" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="17" t="inlineStr">
@@ -1392,6 +1498,9 @@
           <t>ALCANCE</t>
         </is>
       </c>
+      <c r="B4" s="22" t="n"/>
+      <c r="C4" s="22" t="n"/>
+      <c r="D4" s="23" t="n"/>
     </row>
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
@@ -1399,6 +1508,9 @@
           <t>Login · Registro de viajeros · Módulo Menores · Módulo Vehículos · Revisión SAG · Revisión PDI · Vista Integrada · Autorización Final · Informes estadísticos</t>
         </is>
       </c>
+      <c r="B5" s="22" t="n"/>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="23" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
@@ -1406,6 +1518,9 @@
           <t>NORMAS</t>
         </is>
       </c>
+      <c r="B6" s="22" t="n"/>
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="23" t="n"/>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -1414,6 +1529,9 @@
 ISO/IEC 9126 — modelo de características de calidad aplicado al prototipo</t>
         </is>
       </c>
+      <c r="B7" s="22" t="n"/>
+      <c r="C7" s="22" t="n"/>
+      <c r="D7" s="23" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
@@ -1421,6 +1539,9 @@
           <t>ESTRATEGIA</t>
         </is>
       </c>
+      <c r="B8" s="22" t="n"/>
+      <c r="C8" s="22" t="n"/>
+      <c r="D8" s="23" t="n"/>
     </row>
     <row r="9" ht="56" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
@@ -1430,6 +1551,9 @@
 Ambiente: prototipo navegable en Figma — navegador Chrome</t>
         </is>
       </c>
+      <c r="B9" s="22" t="n"/>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="23" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="17" t="inlineStr">
@@ -1437,6 +1561,9 @@
           <t>CRITERIOS</t>
         </is>
       </c>
+      <c r="B10" s="22" t="n"/>
+      <c r="C10" s="22" t="n"/>
+      <c r="D10" s="23" t="n"/>
     </row>
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
@@ -1445,6 +1572,9 @@
 FAIL: resultado difiere del esperado o el caso no puede ejecutarse</t>
         </is>
       </c>
+      <c r="B11" s="22" t="n"/>
+      <c r="C11" s="22" t="n"/>
+      <c r="D11" s="23" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="18" t="inlineStr">

</xml_diff>